<commit_message>
fold the supplements into their figures and name every file after its step
</commit_message>
<xml_diff>
--- a/02_HRvLR/03_Module_Contrasts/c_data/module_contrasts.xlsx
+++ b/02_HRvLR/03_Module_Contrasts/c_data/module_contrasts.xlsx
@@ -253,7 +253,7 @@
     <t>modules</t>
   </si>
   <si>
-    <t>01_Processing/06_Module_Building/c_data/modules.rds</t>
+    <t>01_Processing/06_Module_Building/c_data/module_building.rds</t>
   </si>
   <si>
     <t>32c36eae09056636394bdb0714dd608a</t>
@@ -262,7 +262,7 @@
     <t>fit</t>
   </si>
   <si>
-    <t>02_HRvLR/01_Protein_Contrasts/c_data/fit.rds</t>
+    <t>02_HRvLR/01_Protein_Contrasts/c_data/protein_contrasts.rds</t>
   </si>
   <si>
     <t>d02188e2b55c48f0bc3a965dd3e44bf3</t>

</xml_diff>